<commit_message>
Added more excel formatting
</commit_message>
<xml_diff>
--- a/test_worksheet.xlsx
+++ b/test_worksheet.xlsx
@@ -8,15 +8,70 @@
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+  <si>
+    <t>Finances</t>
+  </si>
+  <si>
+    <t>filler variable</t>
+  </si>
+  <si>
+    <t>Jan</t>
+  </si>
+  <si>
+    <t>Feb</t>
+  </si>
+  <si>
+    <t>Mar</t>
+  </si>
+  <si>
+    <t>April</t>
+  </si>
+  <si>
+    <t>May</t>
+  </si>
+  <si>
+    <t>June</t>
+  </si>
+  <si>
+    <t>July</t>
+  </si>
+  <si>
+    <t>Aug</t>
+  </si>
+  <si>
+    <t>Sept</t>
+  </si>
+  <si>
+    <t>Oct</t>
+  </si>
+  <si>
+    <t>Nov</t>
+  </si>
+  <si>
+    <t>Dec</t>
+  </si>
+  <si>
+    <t>Total Yearly</t>
+  </si>
+  <si>
+    <t>Averages</t>
+  </si>
+  <si>
+    <t>Income</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="1">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -24,13 +79,48 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <u/>
+      <sz val="15"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="15"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFB3FF79"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF46C732"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -45,8 +135,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -341,18 +434,86 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
+  <dimension ref="A1:O3"/>
   <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="15.7109375" customWidth="1"/>
+    <col min="2" max="13" width="10.7109375" customWidth="1"/>
+    <col min="14" max="15" width="15.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:15">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15">
+      <c r="B2" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="M2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="N2" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="O2" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15">
+      <c r="A3" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3"/>
+      <c r="G3" s="3"/>
+      <c r="H3" s="3"/>
+      <c r="I3" s="3"/>
+      <c r="J3" s="3"/>
+      <c r="K3" s="3"/>
+      <c r="L3" s="3"/>
+      <c r="M3" s="3"/>
+      <c r="N3" s="3"/>
+      <c r="O3" s="3"/>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
added more category row labels
</commit_message>
<xml_diff>
--- a/test_worksheet.xlsx
+++ b/test_worksheet.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="21">
   <si>
     <t>Finances</t>
   </si>
@@ -62,6 +62,21 @@
   </si>
   <si>
     <t>Income</t>
+  </si>
+  <si>
+    <t>Food</t>
+  </si>
+  <si>
+    <t>Toiletries</t>
+  </si>
+  <si>
+    <t>Income Total</t>
+  </si>
+  <si>
+    <t>Expenses</t>
+  </si>
+  <si>
+    <t>Total Expenses</t>
   </si>
 </sst>
 </file>
@@ -71,7 +86,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd-mm-yyyy"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -102,8 +117,16 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -122,6 +145,18 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1551BA"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF5352E"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -135,12 +170,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -435,10 +474,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O3"/>
+  <dimension ref="A1:O8"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="15.7109375" customWidth="1"/>
+    <col min="1" max="1" width="18.7109375" customWidth="1"/>
     <col min="2" max="13" width="10.7109375" customWidth="1"/>
     <col min="14" max="15" width="15.7109375" customWidth="1"/>
   </cols>
@@ -517,6 +556,45 @@
       <c r="N3" s="4"/>
       <c r="O3" s="4"/>
     </row>
+    <row r="4" spans="1:15">
+      <c r="A4" s="5" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15">
+      <c r="A5" s="5" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15">
+      <c r="A6" s="6" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15">
+      <c r="A7" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7" s="7"/>
+      <c r="C7" s="7"/>
+      <c r="D7" s="7"/>
+      <c r="E7" s="7"/>
+      <c r="F7" s="7"/>
+      <c r="G7" s="7"/>
+      <c r="H7" s="7"/>
+      <c r="I7" s="7"/>
+      <c r="J7" s="7"/>
+      <c r="K7" s="7"/>
+      <c r="L7" s="7"/>
+      <c r="M7" s="7"/>
+      <c r="N7" s="7"/>
+      <c r="O7" s="7"/>
+    </row>
+    <row r="8" spans="1:15">
+      <c r="A8" s="8" t="s">
+        <v>20</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
added income total formulas
</commit_message>
<xml_diff>
--- a/test_worksheet.xlsx
+++ b/test_worksheet.xlsx
@@ -602,6 +602,62 @@
       <c r="A6" s="7" t="s">
         <v>18</v>
       </c>
+      <c r="B6" s="6">
+        <f>SUM(B4, B5)</f>
+        <v>0</v>
+      </c>
+      <c r="C6" s="6">
+        <f>SUM(C4, C5)</f>
+        <v>0</v>
+      </c>
+      <c r="D6" s="6">
+        <f>SUM(D4, D5)</f>
+        <v>0</v>
+      </c>
+      <c r="E6" s="6">
+        <f>SUM(E4, E5)</f>
+        <v>0</v>
+      </c>
+      <c r="F6" s="6">
+        <f>SUM(F4, F5)</f>
+        <v>0</v>
+      </c>
+      <c r="G6" s="6">
+        <f>SUM(G4, G5)</f>
+        <v>0</v>
+      </c>
+      <c r="H6" s="6">
+        <f>SUM(H4, H5)</f>
+        <v>0</v>
+      </c>
+      <c r="I6" s="6">
+        <f>SUM(I4, I5)</f>
+        <v>0</v>
+      </c>
+      <c r="J6" s="6">
+        <f>SUM(J4, J5)</f>
+        <v>0</v>
+      </c>
+      <c r="K6" s="6">
+        <f>SUM(K4, K5)</f>
+        <v>0</v>
+      </c>
+      <c r="L6" s="6">
+        <f>SUM(L4, L5)</f>
+        <v>0</v>
+      </c>
+      <c r="M6" s="6">
+        <f>SUM(M4, M5)</f>
+        <v>0</v>
+      </c>
+      <c r="N6" s="6">
+        <f>SUM(N4, N5)</f>
+        <v>0</v>
+      </c>
+      <c r="O6" s="6">
+        <f>SUM(O4, O5)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="7" spans="1:15">
       <c r="A7" s="8" t="s">

</xml_diff>

<commit_message>
added percentage savings format
</commit_message>
<xml_diff>
--- a/test_worksheet.xlsx
+++ b/test_worksheet.xlsx
@@ -812,6 +812,62 @@
       <c r="A11" s="11" t="s">
         <v>23</v>
       </c>
+      <c r="B11" s="11">
+        <f>B6/B10</f>
+        <v>0</v>
+      </c>
+      <c r="C11" s="11">
+        <f>C6/C10</f>
+        <v>0</v>
+      </c>
+      <c r="D11" s="11">
+        <f>D6/D10</f>
+        <v>0</v>
+      </c>
+      <c r="E11" s="11">
+        <f>E6/E10</f>
+        <v>0</v>
+      </c>
+      <c r="F11" s="11">
+        <f>F6/F10</f>
+        <v>0</v>
+      </c>
+      <c r="G11" s="11">
+        <f>G6/G10</f>
+        <v>0</v>
+      </c>
+      <c r="H11" s="11">
+        <f>H6/H10</f>
+        <v>0</v>
+      </c>
+      <c r="I11" s="11">
+        <f>I6/I10</f>
+        <v>0</v>
+      </c>
+      <c r="J11" s="11">
+        <f>J6/J10</f>
+        <v>0</v>
+      </c>
+      <c r="K11" s="11">
+        <f>K6/K10</f>
+        <v>0</v>
+      </c>
+      <c r="L11" s="11">
+        <f>L6/L10</f>
+        <v>0</v>
+      </c>
+      <c r="M11" s="11">
+        <f>M6/M10</f>
+        <v>0</v>
+      </c>
+      <c r="N11" s="11">
+        <f>N6/N10</f>
+        <v>0</v>
+      </c>
+      <c r="O11" s="11">
+        <f>O6/O10</f>
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>